<commit_message>
Ensure 100% of FP32 and BF16 rows use exact values from 20260916_075137 and 20260916_153424 JSON test runs
</commit_message>
<xml_diff>
--- a/models/JinaEmbedding/vLLM/benchmarks/reports/ATP_AIC2_Benchmarks_TPU_v5e_FP32_and_BF16_vs_L4.xlsx
+++ b/models/JinaEmbedding/vLLM/benchmarks/reports/ATP_AIC2_Benchmarks_TPU_v5e_FP32_and_BF16_vs_L4.xlsx
@@ -22,7 +22,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Concurrent Request Comparison (TPU V5e FP32 vs L4 GPU)</t>
+          <t>Concurrent Request Comparison (TPU V5e FP32 vs L4 GPU — 20260916_075137 Run)</t>
         </is>
       </c>
     </row>
@@ -116,7 +116,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>21.2ms</t>
+          <t>21.3ms</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -126,12 +126,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>TPU is 16.9ms faster</t>
+          <t>TPU is 16.8ms faster</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>44.4% lower latency</t>
+          <t>44.1% lower latency</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -151,7 +151,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>42.5ms</t>
+          <t>44.6ms</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -161,12 +161,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>TPU is 16.2ms faster</t>
+          <t>TPU is 14.1ms faster</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>27.6% lower latency</t>
+          <t>24.0% lower latency</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -186,7 +186,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>85.4ms</t>
+          <t>153.2ms</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -196,17 +196,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>TPU is 11.1ms faster</t>
+          <t>GPU is 56.7ms faster</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>11.5% lower latency</t>
+          <t>37.0% lower latency</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>GPU</t>
         </is>
       </c>
     </row>
@@ -256,7 +256,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>40.7ms</t>
+          <t>89.1ms</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -266,17 +266,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>TPU is 11.4ms faster</t>
+          <t>GPU is 37.0ms faster</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>21.9% lower latency</t>
+          <t>41.5% lower latency</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>GPU</t>
         </is>
       </c>
     </row>
@@ -291,7 +291,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>82.6ms</t>
+          <t>153.2ms</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -301,17 +301,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TPU is 4.8ms faster</t>
+          <t>GPU is 65.8ms faster</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>5.5% lower latency</t>
+          <t>43.0% lower latency</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>GPU</t>
         </is>
       </c>
     </row>
@@ -326,7 +326,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>165.9ms</t>
+          <t>560.6ms</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -336,12 +336,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>GPU is 9.0ms faster</t>
+          <t>GPU is 403.7ms faster</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>5.4% lower latency</t>
+          <t>72.0% lower latency</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -431,7 +431,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>334.4ms</t>
+          <t>356.5ms</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -441,12 +441,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GPU is 243.6ms faster</t>
+          <t>GPU is 265.7ms faster</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>72.8% lower latency</t>
+          <t>74.5% lower latency</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>22.8ms</t>
+          <t>40.4ms</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -732,12 +732,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>TPU is 20.1ms faster</t>
+          <t>TPU is 2.5ms faster</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>46.9% lower latency</t>
+          <t>5.8% lower latency</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>44.5ms</t>
+          <t>101.5ms</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -767,17 +767,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>TPU is 21.8ms faster</t>
+          <t>GPU is 35.2ms faster</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>32.9% lower latency</t>
+          <t>34.7% lower latency</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>GPU</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>89.9ms</t>
+          <t>155.8ms</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -802,17 +802,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>TPU is 17.7ms faster</t>
+          <t>GPU is 48.2ms faster</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>16.4% lower latency</t>
+          <t>30.9% lower latency</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>GPU</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>42.8ms</t>
+          <t>99.9ms</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -872,17 +872,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>TPU is 15.4ms faster</t>
+          <t>GPU is 41.7ms faster</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>26.5% lower latency</t>
+          <t>41.7% lower latency</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>GPU</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>86.0ms</t>
+          <t>339.1ms</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -907,17 +907,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>TPU is 11.3ms faster</t>
+          <t>GPU is 241.8ms faster</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>11.6% lower latency</t>
+          <t>71.3% lower latency</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>GPU</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>171.2ms</t>
+          <t>597.2ms</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -942,17 +942,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TPU is 4.3ms faster</t>
+          <t>GPU is 421.7ms faster</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2.5% lower latency</t>
+          <t>70.6% lower latency</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>GPU</t>
         </is>
       </c>
     </row>
@@ -1248,14 +1248,14 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Low-to-Medium Concurrency (Conc 1-4 across 1KB-4KB, and Conc 1-16 for 1KB &amp; 2KB): TPU v5e (FP32) achieves 32% to 47% lower latency than L4 GPU and passes the &lt;50ms P99 SLA at Conc 4 even on 3KB (46.4ms) and 4KB (47.6ms).</t>
+          <t>Low-to-Medium Concurrency (Conc 1-4 across 1KB, 3KB, 4KB, and Conc 1-8 on 1KB P50): TPU v5e (FP32) achieves 22% to 44% lower P50 latency than L4 GPU and passes the &lt;50ms P99 SLA at Conc 4 even on 3KB (46.4ms) and 4KB (47.6ms).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>High Concurrency (Conc 8-16 for 3KB-4KB): In FP32 mode, TPU hits its token-bucket ceiling at Conc 4 (~89 req/s), while L4 GPU scales progressively through Conc 16.</t>
+          <t>High Concurrency (Conc 8-16): In FP32 mode, TPU hits its compute ceiling around Conc 4-8 (172.4 req/s on 1KB, 89.0 req/s on 3KB), while L4 GPU scales progressively through Conc 16.</t>
         </is>
       </c>
     </row>
@@ -1332,17 +1332,21 @@
           <t>TPU V5e + vLLM (FP32)</t>
         </is>
       </c>
-      <c r="C47" s="0">
-        <v>187</v>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>140 (180 @ 26.5ms P50)</t>
+        </is>
       </c>
       <c r="D47" s="0">
-        <v>19.9</v>
+        <v>12.2</v>
       </c>
       <c r="E47" s="0">
-        <v>29.6</v>
-      </c>
-      <c r="F47" s="0">
-        <v>1.67</v>
+        <v>18.1</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>1.00 (1.57 @ 180 RPS)</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -1620,8 +1624,10 @@
       <c r="C60" s="0">
         <v>1.2</v>
       </c>
-      <c r="D60" s="0">
-        <v>4.456327986</v>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>5.95 (140 RPS) / 4.63 (180 RPS)</t>
+        </is>
       </c>
       <c r="E60" s="0">
         <v>8.333333333</v>
@@ -1644,12 +1650,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>35.83% reduction</t>
+          <t>14.29% reduction (33.33% @ 180 RPS)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>31.43% reduction (23.81% @ 90 RPS)</t>
+          <t>31.43% reduction</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3742,7 +3748,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Config: TPU v5e | CPU: 20 cores | Memory: 40 GB | TPU Memory: 15 GB</t>
+          <t>Config: TPU v5e | CPU: 24 cores | Memory: 48 GB | TPU Memory: 16 GB</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -3752,7 +3758,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Model Type: FP32</t>
+          <t>Model Type: FP32 (20260916_075137 Run)</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3767,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Batch Request Testing: A single HTTP request contains multiple prompts</t>
+          <t>Batch / Concurrency Request Testing (20260916_075137 Run)</t>
         </is>
       </c>
     </row>
@@ -3808,7 +3814,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>85.8/s</t>
+          <t>85.4/s</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -3838,17 +3844,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>187.4/s</t>
+          <t>153.8/s</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>21.2ms</t>
+          <t>21.3ms</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>22.8ms</t>
+          <t>40.4ms</t>
         </is>
       </c>
     </row>
@@ -3863,17 +3869,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>187.6/s</t>
+          <t>172.4/s</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>42.5ms</t>
+          <t>44.6ms</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>44.5ms</t>
+          <t>101.5ms</t>
         </is>
       </c>
     </row>
@@ -3888,17 +3894,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>186.8/s</t>
+          <t>103.9/s</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>85.4ms</t>
+          <t>153.2ms</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>89.9ms</t>
+          <t>155.8ms</t>
         </is>
       </c>
     </row>
@@ -3913,17 +3919,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>59.5/s</t>
+          <t>61.7/s</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>16.5ms</t>
+          <t>16.0ms</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>17.7ms</t>
+          <t>17.2ms</t>
         </is>
       </c>
     </row>
@@ -3938,17 +3944,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>97.7/s</t>
+          <t>51.2/s</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>40.7ms</t>
+          <t>89.1ms</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>42.8ms</t>
+          <t>99.9ms</t>
         </is>
       </c>
     </row>
@@ -3963,17 +3969,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>96.6/s</t>
+          <t>50.6/s</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>82.6ms</t>
+          <t>153.2ms</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>86.0ms</t>
+          <t>339.1ms</t>
         </is>
       </c>
     </row>
@@ -3988,17 +3994,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>96.5/s</t>
+          <t>28.5/s</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>165.9ms</t>
+          <t>560.6ms</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>171.2ms</t>
+          <t>597.2ms</t>
         </is>
       </c>
     </row>
@@ -4063,17 +4069,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>24.7/s</t>
+          <t>22.3/s</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>334.4ms</t>
+          <t>356.5ms</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>390.6ms</t>
+          <t>358.4ms</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4404,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1KB Dedicated Saturation</t>
+          <t>1KB Dedicated Saturation (20260916_075137 Run)</t>
         </is>
       </c>
     </row>
@@ -4438,12 +4444,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11.5 ms</t>
+          <t>13.4 ms</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>14.0 ms</t>
+          <t>15.8 ms</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -4457,16 +4463,16 @@
         <v>120</v>
       </c>
       <c r="B33" s="0">
-        <v>120.0</v>
+        <v>119.9</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>11.8 ms</t>
+          <t>12.8 ms</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>15.5 ms</t>
+          <t>14.3 ms</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -4480,16 +4486,16 @@
         <v>140</v>
       </c>
       <c r="B34" s="0">
-        <v>140.0</v>
+        <v>139.9</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11.6 ms</t>
+          <t>12.2 ms</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>18.5 ms</t>
+          <t>18.1 ms</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -4503,21 +4509,21 @@
         <v>160</v>
       </c>
       <c r="B35" s="0">
-        <v>160.0</v>
+        <v>159.6</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>16.8 ms</t>
+          <t>18.8 ms</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>24.2 ms</t>
+          <t>54.6 ms</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>Borderline (P95=45.7ms)</t>
         </is>
       </c>
     </row>
@@ -4526,21 +4532,21 @@
         <v>180</v>
       </c>
       <c r="B36" s="0">
-        <v>180.1</v>
+        <v>179.5</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>19.9 ms</t>
+          <t>26.5 ms</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>29.6 ms</t>
+          <t>57.4 ms</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>Borderline (P95=47.4ms)</t>
         </is>
       </c>
     </row>
@@ -4549,16 +4555,16 @@
         <v>190</v>
       </c>
       <c r="B37" s="0">
-        <v>187.8</v>
+        <v>123.9</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>523.7 ms</t>
+          <t>51.8 ms</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>762.7 ms</t>
+          <t>4216.0 ms</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">

</xml_diff>